<commit_message>
Own 5 V for the pedal, CAN terminator option, Mini-Fit Jr aux connector
- Pedal supply C15 (APS_PS_5V) now from the second power module M8's protected 5 V; C16 sensor 5 V stays on M14. M8 fed like M14 (+12V_RAW, +12V_IGN, +12V_BACK_UP, PWR_EN). Open JP11 falls back to +5VAS; M8 power-good on pad P32.
- CAN: M1 terminates internally (R100 120R); WBO has none. R52 120R (DNP) at the aux connector for an external bus end.
- J3 aux connector, Molex Mini-Fit Jr 5566-14A 2x7 vertical (39281143): +12 V via F6 0.5 A PTC, +5 V sensor via F7 50 mA PTC, sensor ground, AUX_IN1-3 (launch/2-step, map switch, spare), AUX_AN1 (IN_RES2), AUX_AN2 (IN_AT2, shared with the FPCU status option), two low-side outputs, CAN H/L, 2x GND. Symbol and footprint from KiCad 8.0.7 libs; footprint copied into STI.pretty.

Verified: 104 planned nets match the netlist; whole-netlist diff clean; ERC errors 155 -> 148, no new types; pinout check 99 OK.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/STI2004-pinout-check.xlsx
+++ b/documents/STI2004-pinout-check.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="561">
   <si>
     <t>Status</t>
   </si>
@@ -367,7 +367,7 @@
     <t>+12V_IGN</t>
   </si>
   <si>
-    <t>M14.IN_VIGN_V2</t>
+    <t>M14.IN_VIGN_V2; M8.IN_VIGN_V2</t>
   </si>
   <si>
     <t>D16</t>
@@ -733,22 +733,25 @@
     <t>APS_PS_5V</t>
   </si>
   <si>
+    <t>JP11.1_1; M8.5VP_V4</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>Sensor power supply</t>
+  </si>
+  <si>
+    <t>5v OUT SENSOR_PS_5V</t>
+  </si>
+  <si>
+    <t>SENSOR_PS_5V</t>
+  </si>
+  <si>
     <t>+5VAS</t>
   </si>
   <si>
-    <t>M14.5VP_V4</t>
-  </si>
-  <si>
-    <t>C16</t>
-  </si>
-  <si>
-    <t>Sensor power supply</t>
-  </si>
-  <si>
-    <t>5v OUT SENSOR_PS_5V</t>
-  </si>
-  <si>
-    <t>SENSOR_PS_5V</t>
+    <t>F7 -&gt; AUX_5V -&gt; J3.Pin_3_3; JP11.2_2; M14.5VP_V4</t>
   </si>
   <si>
     <t>Feeds throttle TPS; MAP; TGV sensors</t>
@@ -949,7 +952,7 @@
     <t>GND_SENSOR</t>
   </si>
   <si>
-    <t>JP8.1_1; JP9.1_1</t>
+    <t>J3.Pin_4_4; JP8.1_1; JP9.1_1</t>
   </si>
   <si>
     <t>C32</t>
@@ -1177,7 +1180,7 @@
     <t>+12V_BACK_UP</t>
   </si>
   <si>
-    <t>M14.V12_PERM_V1</t>
+    <t>M14.V12_PERM_V1; M8.V12_PERM_V1</t>
   </si>
   <si>
     <t>Ignition OFF: 10-13</t>
@@ -2720,7 +2723,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="16" ht="30.75">
+    <row r="16" ht="71.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -3924,17 +3927,17 @@
         <v>238</v>
       </c>
       <c r="L47" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="M47" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="M47" s="4" t="s">
-        <v>240</v>
-      </c>
       <c r="N47" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O47" s="4"/>
     </row>
-    <row r="48" ht="71.25">
+    <row r="48" ht="98.25">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -3945,10 +3948,10 @@
         <v>16</v>
       </c>
       <c r="D48" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="E48" s="4" t="s">
         <v>241</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>242</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>237</v>
@@ -3963,22 +3966,22 @@
         <v>75</v>
       </c>
       <c r="J48" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="K48" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="K48" s="4" t="s">
+      <c r="L48" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="L48" s="4" t="s">
-        <v>239</v>
-      </c>
       <c r="M48" s="4" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="N48" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O48" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="49" ht="57.75">
@@ -3992,34 +3995,34 @@
         <v>17</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I49" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L49" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="M49" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="N49" s="4" t="s">
         <v>3</v>
@@ -4037,34 +4040,34 @@
         <v>18</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="I50" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L50" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="M50" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="N50" s="4" t="s">
         <v>3</v>
@@ -4082,7 +4085,7 @@
         <v>19</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>130</v>
@@ -4111,32 +4114,32 @@
         <v>20</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I52" s="4" t="s">
         <v>42</v>
       </c>
       <c r="J52" s="4"/>
       <c r="K52" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="L52" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="M52" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="N52" s="4" t="s">
         <v>3</v>
@@ -4154,19 +4157,19 @@
         <v>21</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>42</v>
@@ -4191,19 +4194,19 @@
         <v>22</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I54" s="4" t="s">
         <v>42</v>
@@ -4211,10 +4214,10 @@
       <c r="J54" s="4"/>
       <c r="K54" s="4"/>
       <c r="L54" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="M54" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="N54" s="4" t="s">
         <v>3</v>
@@ -4232,32 +4235,32 @@
         <v>23</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>152</v>
       </c>
       <c r="J55" s="4"/>
       <c r="K55" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L55" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="M55" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="N55" s="4" t="s">
         <v>3</v>
@@ -4275,7 +4278,7 @@
         <v>24</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>130</v>
@@ -4304,13 +4307,13 @@
         <v>25</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G57" s="4">
         <v>2.8</v>
@@ -4323,13 +4326,13 @@
       </c>
       <c r="J57" s="4"/>
       <c r="K57" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L57" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="M57" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="N57" s="4" t="s">
         <v>3</v>
@@ -4347,34 +4350,34 @@
         <v>26</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I58" s="4" t="s">
         <v>75</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K58" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L58" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="M58" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="N58" s="4" t="s">
         <v>3</v>
@@ -4392,34 +4395,34 @@
         <v>27</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I59" s="4" t="s">
         <v>75</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K59" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L59" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="M59" s="4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="N59" s="4" t="s">
         <v>3</v>
@@ -4437,34 +4440,34 @@
         <v>28</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I60" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K60" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L60" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="M60" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="N60" s="4" t="s">
         <v>3</v>
@@ -4482,34 +4485,34 @@
         <v>29</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I61" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K61" s="4" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L61" s="4" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="M61" s="4" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="N61" s="4" t="s">
         <v>3</v>
@@ -4527,7 +4530,7 @@
         <v>30</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>130</v>
@@ -4556,10 +4559,10 @@
         <v>31</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>48</v>
@@ -4578,10 +4581,10 @@
         <v>43</v>
       </c>
       <c r="L63" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="M63" s="4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="N63" s="4" t="s">
         <v>3</v>
@@ -4599,10 +4602,10 @@
         <v>32</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>172</v>
@@ -4642,10 +4645,10 @@
         <v>33</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F65" s="4" t="s">
         <v>172</v>
@@ -4685,10 +4688,10 @@
         <v>34</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F66" s="4" t="s">
         <v>48</v>
@@ -4703,16 +4706,16 @@
         <v>49</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K66" s="4" t="s">
         <v>43</v>
       </c>
       <c r="L66" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="M66" s="4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="N66" s="4" t="s">
         <v>3</v>
@@ -4730,10 +4733,10 @@
         <v>35</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F67" s="4" t="s">
         <v>48</v>
@@ -4752,16 +4755,16 @@
         <v>43</v>
       </c>
       <c r="L67" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="M67" s="4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="N67" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O67" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="68" ht="44.25">
@@ -4769,16 +4772,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C68" s="4">
         <v>1</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F68" s="4" t="s">
         <v>41</v>
@@ -4812,25 +4815,25 @@
         <v>68</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C69" s="4">
         <v>2</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I69" s="4" t="s">
         <v>152</v>
@@ -4838,10 +4841,10 @@
       <c r="J69" s="4"/>
       <c r="K69" s="4"/>
       <c r="L69" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="M69" s="4" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="N69" s="4" t="s">
         <v>3</v>
@@ -4853,13 +4856,13 @@
         <v>69</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C70" s="4">
         <v>3</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>130</v>
@@ -4882,16 +4885,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C71" s="4">
         <v>4</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F71" s="4" t="s">
         <v>41</v>
@@ -4925,19 +4928,19 @@
         <v>71</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C72" s="4">
         <v>5</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G72" s="5">
         <v>46308</v>
@@ -4949,13 +4952,13 @@
         <v>75</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K72" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="L72" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M72" s="4" t="s">
         <v>44</v>
@@ -4970,19 +4973,19 @@
         <v>72</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C73" s="4">
         <v>6</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G73" s="5">
         <v>46308</v>
@@ -4994,13 +4997,13 @@
         <v>75</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K73" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="L73" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M73" s="4" t="s">
         <v>44</v>
@@ -5015,13 +5018,13 @@
         <v>73</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C74" s="4">
         <v>7</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>130</v>
@@ -5044,40 +5047,40 @@
         <v>74</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C75" s="4">
         <v>8</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G75" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="I75" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J75" s="4" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K75" s="4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="L75" s="4" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="M75" s="4" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="N75" s="4" t="s">
         <v>3</v>
@@ -5089,40 +5092,40 @@
         <v>75</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C76" s="4">
         <v>9</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G76" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="I76" s="4" t="s">
         <v>49</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K76" s="4" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L76" s="4" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="M76" s="4" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="N76" s="4" t="s">
         <v>3</v>
@@ -5134,40 +5137,40 @@
         <v>76</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C77" s="4">
         <v>10</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G77" s="4">
         <v>0</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>152</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="K77" s="4" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="L77" s="4" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="M77" s="4" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="N77" s="4" t="s">
         <v>3</v>
@@ -5179,13 +5182,13 @@
         <v>77</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C78" s="4">
         <v>11</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>130</v>
@@ -5208,16 +5211,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C79" s="4">
         <v>12</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F79" s="4" t="s">
         <v>41</v>
@@ -5251,13 +5254,13 @@
         <v>79</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C80" s="4">
         <v>13</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E80" s="4" t="s">
         <v>130</v>
@@ -5280,13 +5283,13 @@
         <v>80</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C81" s="4">
         <v>14</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E81" s="4" t="s">
         <v>130</v>
@@ -5309,19 +5312,19 @@
         <v>81</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C82" s="4">
         <v>15</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G82" s="4">
         <v>0</v>
@@ -5330,23 +5333,23 @@
         <v>65</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J82" s="4"/>
       <c r="K82" s="4" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="L82" s="4" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="M82" s="4" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="N82" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O82" s="4" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="83" ht="57.75">
@@ -5354,19 +5357,19 @@
         <v>82</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C83" s="4">
         <v>16</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G83" s="4">
         <v>0</v>
@@ -5379,13 +5382,13 @@
       </c>
       <c r="J83" s="4"/>
       <c r="K83" s="4" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="L83" s="4" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="M83" s="4" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="N83" s="4" t="s">
         <v>3</v>
@@ -5397,19 +5400,19 @@
         <v>83</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C84" s="4">
         <v>17</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G84" s="4">
         <v>0</v>
@@ -5422,13 +5425,13 @@
       </c>
       <c r="J84" s="4"/>
       <c r="K84" s="4" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="L84" s="4" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="M84" s="4" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="N84" s="4" t="s">
         <v>3</v>
@@ -5440,19 +5443,19 @@
         <v>84</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C85" s="4">
         <v>18</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G85" s="4">
         <v>0</v>
@@ -5465,37 +5468,37 @@
       </c>
       <c r="J85" s="4"/>
       <c r="K85" s="4" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="L85" s="4" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M85" s="4" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="N85" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O85" s="4"/>
     </row>
-    <row r="86" ht="44.25">
+    <row r="86" ht="71.25">
       <c r="A86" s="4">
         <v>85</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C86" s="4">
         <v>19</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G86" s="5">
         <v>46308</v>
@@ -5508,19 +5511,19 @@
       </c>
       <c r="J86" s="4"/>
       <c r="K86" s="4" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="L86" s="4" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="M86" s="4" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="N86" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O86" s="4" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="87" ht="30.75">
@@ -5528,13 +5531,13 @@
         <v>86</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C87" s="4">
         <v>20</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E87" s="4" t="s">
         <v>130</v>
@@ -5557,13 +5560,13 @@
         <v>87</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C88" s="4">
         <v>21</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E88" s="4" t="s">
         <v>130</v>
@@ -5586,19 +5589,19 @@
         <v>88</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C89" s="4">
         <v>22</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G89" s="4">
         <v>0</v>
@@ -5610,7 +5613,7 @@
         <v>152</v>
       </c>
       <c r="J89" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="K89" s="4" t="s">
         <v>140</v>
@@ -5619,7 +5622,7 @@
         <v>140</v>
       </c>
       <c r="M89" s="4" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="N89" s="4" t="s">
         <v>3</v>
@@ -5631,13 +5634,13 @@
         <v>89</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C90" s="4">
         <v>23</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E90" s="4" t="s">
         <v>130</v>
@@ -5660,44 +5663,44 @@
         <v>90</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C91" s="4">
         <v>24</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F91" s="4" t="s">
         <v>124</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="I91" s="4" t="s">
         <v>75</v>
       </c>
       <c r="J91" s="4"/>
       <c r="K91" s="4" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L91" s="4" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="M91" s="4" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="N91" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O91" s="4" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="92" ht="57.75">
@@ -5705,38 +5708,38 @@
         <v>91</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C92" s="4">
         <v>25</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F92" s="4" t="s">
         <v>124</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="I92" s="4" t="s">
         <v>75</v>
       </c>
       <c r="J92" s="4"/>
       <c r="K92" s="4" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="L92" s="4" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="M92" s="4" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="N92" s="4" t="s">
         <v>3</v>
@@ -5748,44 +5751,44 @@
         <v>92</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C93" s="4">
         <v>26</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="I93" s="4" t="s">
         <v>75</v>
       </c>
       <c r="J93" s="4"/>
       <c r="K93" s="4" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="L93" s="4" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="M93" s="4" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="N93" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O93" s="4" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="94" ht="125.25">
@@ -5793,40 +5796,40 @@
         <v>93</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C94" s="4">
         <v>27</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="I94" s="4" t="s">
         <v>152</v>
       </c>
       <c r="J94" s="4" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="K94" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="L94" s="4" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="M94" s="4" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="N94" s="4" t="s">
         <v>3</v>
@@ -5838,13 +5841,13 @@
         <v>94</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C95" s="4">
         <v>28</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E95" s="4" t="s">
         <v>130</v>
@@ -5867,13 +5870,13 @@
         <v>95</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C96" s="4">
         <v>29</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E96" s="4" t="s">
         <v>130</v>
@@ -5896,13 +5899,13 @@
         <v>96</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C97" s="4">
         <v>30</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E97" s="4" t="s">
         <v>130</v>
@@ -5925,16 +5928,16 @@
         <v>97</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C98" s="4">
         <v>31</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F98" s="4" t="s">
         <v>172</v>
@@ -5968,13 +5971,13 @@
         <v>98</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C99" s="4">
         <v>32</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E99" s="4" t="s">
         <v>130</v>
@@ -5997,25 +6000,25 @@
         <v>99</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C100" s="4">
         <v>33</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F100" s="4" t="s">
         <v>124</v>
       </c>
       <c r="G100" s="4" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="H100" s="4" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="I100" s="4" t="s">
         <v>125</v>
@@ -6023,16 +6026,16 @@
       <c r="J100" s="4"/>
       <c r="K100" s="4"/>
       <c r="L100" s="4" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M100" s="4" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="N100" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O100" s="4" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="101" ht="30.75">
@@ -6040,13 +6043,13 @@
         <v>100</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C101" s="4">
         <v>34</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E101" s="4" t="s">
         <v>130</v>
@@ -6069,16 +6072,16 @@
         <v>101</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C102" s="4">
         <v>35</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F102" s="4" t="s">
         <v>124</v>
@@ -6094,19 +6097,19 @@
       </c>
       <c r="J102" s="4"/>
       <c r="K102" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="L102" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M102" s="4" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="N102" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O102" s="4" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="103" ht="57.75">
@@ -6114,16 +6117,16 @@
         <v>102</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C103" s="4">
         <v>1</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F103" s="4" t="s">
         <v>87</v>
@@ -6138,16 +6141,16 @@
         <v>49</v>
       </c>
       <c r="J103" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="L103" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="M103" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="N103" s="4" t="s">
         <v>3</v>
@@ -6159,25 +6162,25 @@
         <v>103</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C104" s="4">
         <v>2</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E104" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G104" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H104" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I104" s="4" t="s">
         <v>152</v>
@@ -6185,16 +6188,16 @@
       <c r="J104" s="4"/>
       <c r="K104" s="4"/>
       <c r="L104" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="M104" s="4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="N104" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O104" s="4" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="105" ht="111.75">
@@ -6202,25 +6205,25 @@
         <v>104</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C105" s="4">
         <v>3</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G105" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H105" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I105" s="4" t="s">
         <v>152</v>
@@ -6228,16 +6231,16 @@
       <c r="J105" s="4"/>
       <c r="K105" s="4"/>
       <c r="L105" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="M105" s="4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="N105" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O105" s="4" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="106" ht="30.75">
@@ -6245,13 +6248,13 @@
         <v>105</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C106" s="4">
         <v>4</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E106" s="4" t="s">
         <v>130</v>
@@ -6274,13 +6277,13 @@
         <v>106</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C107" s="4">
         <v>5</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E107" s="4" t="s">
         <v>130</v>
@@ -6303,16 +6306,16 @@
         <v>107</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C108" s="4">
         <v>6</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F108" s="4" t="s">
         <v>41</v>
@@ -6346,16 +6349,16 @@
         <v>108</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C109" s="4">
         <v>7</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F109" s="4" t="s">
         <v>41</v>
@@ -6389,25 +6392,25 @@
         <v>109</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C110" s="4">
         <v>8</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G110" s="4" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H110" s="4" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I110" s="4" t="s">
         <v>75</v>
@@ -6415,10 +6418,10 @@
       <c r="J110" s="4"/>
       <c r="K110" s="4"/>
       <c r="L110" s="4" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M110" s="4" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="N110" s="4" t="s">
         <v>3</v>
@@ -6430,25 +6433,25 @@
         <v>110</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C111" s="4">
         <v>9</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E111" s="4" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G111" s="4" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H111" s="4" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I111" s="4" t="s">
         <v>75</v>
@@ -6456,10 +6459,10 @@
       <c r="J111" s="4"/>
       <c r="K111" s="4"/>
       <c r="L111" s="4" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="M111" s="4" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="N111" s="4" t="s">
         <v>3</v>
@@ -6471,25 +6474,25 @@
         <v>111</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C112" s="4">
         <v>10</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G112" s="4" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H112" s="4" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I112" s="4" t="s">
         <v>75</v>
@@ -6497,10 +6500,10 @@
       <c r="J112" s="4"/>
       <c r="K112" s="4"/>
       <c r="L112" s="4" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M112" s="4" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="N112" s="4" t="s">
         <v>3</v>
@@ -6512,25 +6515,25 @@
         <v>112</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C113" s="4">
         <v>11</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G113" s="4" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H113" s="4" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I113" s="4" t="s">
         <v>75</v>
@@ -6538,10 +6541,10 @@
       <c r="J113" s="4"/>
       <c r="K113" s="4"/>
       <c r="L113" s="4" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="M113" s="4" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="N113" s="4" t="s">
         <v>3</v>
@@ -6553,25 +6556,25 @@
         <v>113</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C114" s="4">
         <v>12</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G114" s="4" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="H114" s="4" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I114" s="4" t="s">
         <v>42</v>
@@ -6579,10 +6582,10 @@
       <c r="J114" s="4"/>
       <c r="K114" s="4"/>
       <c r="L114" s="4" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="M114" s="4" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="N114" s="4" t="s">
         <v>3</v>
@@ -6594,25 +6597,25 @@
         <v>114</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C115" s="4">
         <v>13</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G115" s="4" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="H115" s="4" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I115" s="4" t="s">
         <v>42</v>
@@ -6620,10 +6623,10 @@
       <c r="J115" s="4"/>
       <c r="K115" s="4"/>
       <c r="L115" s="4" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="M115" s="4" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="N115" s="4" t="s">
         <v>3</v>
@@ -6635,38 +6638,38 @@
         <v>115</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C116" s="4">
         <v>14</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G116" s="4" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="H116" s="4" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I116" s="4" t="s">
         <v>42</v>
       </c>
       <c r="J116" s="4"/>
       <c r="K116" s="4" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="L116" s="4" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="M116" s="4" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="N116" s="4" t="s">
         <v>3</v>
@@ -6678,19 +6681,19 @@
         <v>116</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C117" s="4">
         <v>15</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G117" s="4" t="s">
         <v>95</v>
@@ -6704,10 +6707,10 @@
       <c r="J117" s="4"/>
       <c r="K117" s="4"/>
       <c r="L117" s="4" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="M117" s="4" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="N117" s="4" t="s">
         <v>3</v>
@@ -6719,19 +6722,19 @@
         <v>117</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C118" s="4">
         <v>16</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G118" s="4" t="s">
         <v>95</v>
@@ -6745,10 +6748,10 @@
       <c r="J118" s="4"/>
       <c r="K118" s="4"/>
       <c r="L118" s="4" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="M118" s="4" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="N118" s="4" t="s">
         <v>3</v>
@@ -6760,25 +6763,25 @@
         <v>118</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C119" s="4">
         <v>17</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G119" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H119" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I119" s="4" t="s">
         <v>42</v>
@@ -6786,16 +6789,16 @@
       <c r="J119" s="4"/>
       <c r="K119" s="4"/>
       <c r="L119" s="4" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="M119" s="4" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="N119" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O119" s="4" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="120" ht="71.25">
@@ -6803,19 +6806,19 @@
         <v>119</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C120" s="4">
         <v>18</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E120" s="4" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="G120" s="4" t="s">
         <v>81</v>
@@ -6827,13 +6830,13 @@
         <v>49</v>
       </c>
       <c r="J120" s="4" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K120" s="4" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="L120" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M120" s="4" t="s">
         <v>44</v>
@@ -6848,19 +6851,19 @@
         <v>120</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C121" s="4">
         <v>19</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E121" s="4" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="G121" s="4" t="s">
         <v>81</v>
@@ -6872,13 +6875,13 @@
         <v>49</v>
       </c>
       <c r="J121" s="4" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="K121" s="4" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="L121" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M121" s="4" t="s">
         <v>44</v>
@@ -6893,13 +6896,13 @@
         <v>121</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C122" s="4">
         <v>20</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E122" s="4" t="s">
         <v>130</v>
@@ -6922,13 +6925,13 @@
         <v>122</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C123" s="4">
         <v>21</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E123" s="4" t="s">
         <v>130</v>
@@ -6951,36 +6954,36 @@
         <v>123</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C124" s="4">
         <v>22</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E124" s="4" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F124" s="4"/>
       <c r="G124" s="4"/>
       <c r="H124" s="4"/>
       <c r="I124" s="4" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J124" s="4"/>
       <c r="K124" s="4"/>
       <c r="L124" s="4" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="M124" s="4" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="N124" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O124" s="4" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="125" ht="57.75">
@@ -6988,46 +6991,46 @@
         <v>124</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C125" s="4">
         <v>23</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E125" s="4" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="G125" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H125" s="4" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="I125" s="4" t="s">
         <v>42</v>
       </c>
       <c r="J125" s="4" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="K125" s="4" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="L125" s="4" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="M125" s="4" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="N125" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O125" s="4" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="126" ht="57.75">
@@ -7035,25 +7038,25 @@
         <v>125</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C126" s="4">
         <v>24</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E126" s="4" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G126" s="4" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="H126" s="4" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I126" s="4" t="s">
         <v>42</v>
@@ -7072,16 +7075,16 @@
         <v>126</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C127" s="4">
         <v>25</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E127" s="4" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F127" s="4" t="s">
         <v>172</v>
@@ -7098,10 +7101,10 @@
       <c r="J127" s="4"/>
       <c r="K127" s="4"/>
       <c r="L127" s="4" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="M127" s="4" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="N127" s="4" t="s">
         <v>3</v>
@@ -7113,25 +7116,25 @@
         <v>127</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C128" s="4">
         <v>26</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="G128" s="4" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="H128" s="4" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="I128" s="4" t="s">
         <v>42</v>
@@ -7139,16 +7142,16 @@
       <c r="J128" s="4"/>
       <c r="K128" s="4"/>
       <c r="L128" s="4" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="M128" s="4" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="N128" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O128" s="4" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="129" ht="30.75">
@@ -7156,13 +7159,13 @@
         <v>128</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C129" s="4">
         <v>27</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E129" s="4" t="s">
         <v>130</v>
@@ -7185,19 +7188,19 @@
         <v>129</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C130" s="4">
         <v>28</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E130" s="4" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="G130" s="4">
         <v>0</v>
@@ -7209,16 +7212,16 @@
         <v>49</v>
       </c>
       <c r="J130" s="4" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="K130" s="4" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="L130" s="4" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="M130" s="4" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="N130" s="4" t="s">
         <v>3</v>
@@ -7230,19 +7233,19 @@
         <v>130</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C131" s="4">
         <v>29</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="G131" s="4">
         <v>0</v>
@@ -7254,16 +7257,16 @@
         <v>49</v>
       </c>
       <c r="J131" s="4" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="K131" s="4" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="L131" s="4" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="M131" s="4" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="N131" s="4" t="s">
         <v>3</v>
@@ -7275,13 +7278,13 @@
         <v>131</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C132" s="4">
         <v>30</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E132" s="4" t="s">
         <v>130</v>
@@ -7304,13 +7307,13 @@
         <v>132</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C133" s="4">
         <v>31</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>130</v>
@@ -7333,40 +7336,40 @@
         <v>133</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C134" s="4">
         <v>32</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="G134" s="4" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H134" s="4" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I134" s="4" t="s">
         <v>75</v>
       </c>
       <c r="J134" s="4" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="K134" s="4" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="L134" s="4" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="M134" s="4" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="N134" s="4" t="s">
         <v>3</v>
@@ -7378,25 +7381,25 @@
         <v>134</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C135" s="4">
         <v>33</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="G135" s="4" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="H135" s="4" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="I135" s="4" t="s">
         <v>42</v>
@@ -7404,16 +7407,16 @@
       <c r="J135" s="4"/>
       <c r="K135" s="4"/>
       <c r="L135" s="4" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="M135" s="4" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="N135" s="4" t="s">
         <v>3</v>
       </c>
       <c r="O135" s="4" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="136" ht="84.75">
@@ -7421,13 +7424,13 @@
         <v>135</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C136" s="4">
         <v>34</v>
       </c>
       <c r="D136" s="4" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E136" s="4" t="s">
         <v>164</v>
@@ -7438,7 +7441,7 @@
       <c r="G136" s="4"/>
       <c r="H136" s="4"/>
       <c r="I136" s="4" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J136" s="4"/>
       <c r="K136" s="4"/>
@@ -7452,7 +7455,7 @@
         <v>3</v>
       </c>
       <c r="O136" s="4" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
On-board MAP sensor (AlphaX style): U20 MPXHZ6400AC6T1 + C1 100n on +5VA -> M1 IN_MAP3 (S19)
TGV position RH moves from IN_MAP3 to IN_RES2 (S14). J3 pin 8 (was AUX_AN1 on
IN_RES2) is now not connected; P28 is the MAP test pad. External MAP stays on
IN_MAP1. PCB: U20/C1 placed left of M1, DRC 0 errors, unconnected 322.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/STI2004-pinout-check.xlsx
+++ b/documents/STI2004-pinout-check.xlsx
@@ -385,7 +385,7 @@
     <t>OUT_MAIN_RELAY</t>
   </si>
   <si>
-    <t>Q5.D_2</t>
+    <t>U12.D_8</t>
   </si>
   <si>
     <t>Not in the I/O table; wiring diagram shows D17 to the main relay coil</t>
@@ -538,7 +538,7 @@
     <t>OUT_INJ4</t>
   </si>
   <si>
-    <t>Q4.D_2</t>
+    <t>U11.D_6</t>
   </si>
   <si>
     <t>C4</t>
@@ -550,7 +550,7 @@
     <t>OUT_INJ3</t>
   </si>
   <si>
-    <t>Q3.D_2</t>
+    <t>U11.D_8</t>
   </si>
   <si>
     <t>C5</t>
@@ -562,7 +562,7 @@
     <t>OUT_INJ2</t>
   </si>
   <si>
-    <t>Q2.D_2</t>
+    <t>U10.D_6</t>
   </si>
   <si>
     <t>C6</t>
@@ -574,7 +574,7 @@
     <t>OUT_INJ1</t>
   </si>
   <si>
-    <t>Q1.D_2</t>
+    <t>U10.D_8</t>
   </si>
   <si>
     <t>C7</t>
@@ -883,7 +883,7 @@
     <t>IN_TUMBLE_SENSOR_RH</t>
   </si>
   <si>
-    <t>M1.IN_MAP3_S19</t>
+    <t>M1.IN_RES2_S14</t>
   </si>
   <si>
     <t>C28</t>
@@ -988,7 +988,7 @@
     <t>OUT_O2_HEATER_REAR</t>
   </si>
   <si>
-    <t>Q14.D_2</t>
+    <t>Q16.D_2</t>
   </si>
   <si>
     <t>B3</t>
@@ -1096,7 +1096,7 @@
     <t>WI-107</t>
   </si>
   <si>
-    <t>Net-(F1-Pad1)</t>
+    <t>Vehicle connector/IGN4_COIL</t>
   </si>
   <si>
     <t>F1 -&gt; OUT_IGN4 -&gt; M1.IGN4_W8</t>
@@ -1111,7 +1111,7 @@
     <t>Ignition control #3</t>
   </si>
   <si>
-    <t>Net-(F2-Pad1)</t>
+    <t>Vehicle connector/IGN3_COIL</t>
   </si>
   <si>
     <t>F2 -&gt; OUT_IGN3 -&gt; M1.IGN3_W9</t>
@@ -1123,7 +1123,7 @@
     <t>Ignition control #2</t>
   </si>
   <si>
-    <t>Net-(F3-Pad1)</t>
+    <t>Vehicle connector/IGN2_COIL</t>
   </si>
   <si>
     <t>F3 -&gt; OUT_IGN2 -&gt; M1.IGN2_W10</t>
@@ -1135,7 +1135,7 @@
     <t>Ignition control #1</t>
   </si>
   <si>
-    <t>Net-(F4-Pad1)</t>
+    <t>Vehicle connector/IGN1_COIL</t>
   </si>
   <si>
     <t>F4 -&gt; OUT_IGN1 -&gt; M1.IGN1_W11</t>
@@ -1198,7 +1198,7 @@
     <t>OUT_FAN_RELAY_2</t>
   </si>
   <si>
-    <t>Q7.D_2</t>
+    <t>U13.D_8</t>
   </si>
   <si>
     <t>Models with A/C only</t>
@@ -1213,7 +1213,7 @@
     <t>OUT_FAN_RELAY_1</t>
   </si>
   <si>
-    <t>Q6.D_2</t>
+    <t>U12.D_6</t>
   </si>
   <si>
     <t>B26</t>
@@ -1279,7 +1279,7 @@
     <t>OUT_AC_RELAY</t>
   </si>
   <si>
-    <t>Q15.D_2</t>
+    <t>U18.D_8</t>
   </si>
   <si>
     <t>I/O table (EN(STi)-19) prints B133 33; wiring diagram shows B33 to the auto A/C module</t>
@@ -1297,7 +1297,7 @@
     <t>OUT_ELECTRONIC_THROTTE_RELAY</t>
   </si>
   <si>
-    <t>Q8.D_2</t>
+    <t>U13.D_6</t>
   </si>
   <si>
     <t>ON whenever the ignition is ON</t>
@@ -1450,7 +1450,7 @@
     <t>OUT_PURGE_CONTROL</t>
   </si>
   <si>
-    <t>Q12.D_2</t>
+    <t>U15.D_6</t>
   </si>
   <si>
     <t>A15</t>
@@ -1465,7 +1465,7 @@
     <t>OUT_CRUISE_MAIN_LIGHT</t>
   </si>
   <si>
-    <t>Q17.D_2</t>
+    <t>U16.D_8</t>
   </si>
   <si>
     <t>A16</t>
@@ -1477,7 +1477,7 @@
     <t>OUT_CRUISE_SET_LIGHT</t>
   </si>
   <si>
-    <t>Q18.D_2</t>
+    <t>U16.D_6</t>
   </si>
   <si>
     <t>A17</t>
@@ -1489,7 +1489,7 @@
     <t>OUT_MIL</t>
   </si>
   <si>
-    <t>Q13.D_2</t>
+    <t>U17.D_8</t>
   </si>
   <si>
     <t>ON &lt;=1 / OFF 10-14</t>
@@ -1555,7 +1555,7 @@
     <t>OUT_TACH</t>
   </si>
   <si>
-    <t>Q16.D_2; R38.1</t>
+    <t>R38.1; U17.D_6</t>
   </si>
   <si>
     <t>A24</t>
@@ -1612,7 +1612,7 @@
     <t>OUT_VVT_RH-</t>
   </si>
   <si>
-    <t>Q10.D_2</t>
+    <t>U14.D_6</t>
   </si>
   <si>
     <t>A29</t>
@@ -1624,7 +1624,7 @@
     <t>OUT_VVT_LH-</t>
   </si>
   <si>
-    <t>Q11.D_2</t>
+    <t>U15.D_8</t>
   </si>
   <si>
     <t>A30</t>
@@ -1648,7 +1648,7 @@
     <t>OUT_WG</t>
   </si>
   <si>
-    <t>Q9.D_2</t>
+    <t>U14.D_8</t>
   </si>
   <si>
     <t>A33</t>

</xml_diff>